<commit_message>
Fix textarea click issue in matter panel, fix Excel template sample rows
</commit_message>
<xml_diff>
--- a/frontend/MutemoDesk_Matter_Import_Template.xlsx
+++ b/frontend/MutemoDesk_Matter_Import_Template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,8 +78,20 @@
       <color rgb="002E75B6"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +128,11 @@
         <fgColor rgb="00F9FCFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -185,6 +202,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -687,236 +710,236 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>NGM 1</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE-NGM1</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Abigail Munjeya</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Estate Late Itai Sunguro</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr"/>
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Estate / Inheritance</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr"/>
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Awaiting Court</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>NGM appointed as Executor</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>Waiting for appointment of curator for Michael Sunguro</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>24/03/26</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>NGM 2</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE-NGM2</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Daphne Musengi</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Divorce proceedings</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Vengai Musengi</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Matrimonial / Divorce</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Awaiting Client</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>Matter removed from unopposed roll, dismissed</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>Awaiting further instructions and payment of fees</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J7" s="15" t="inlineStr">
         <is>
           <t>18/01/26</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>NGM 3</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE-NGM3</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Kudzai Madzingira</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Application for declarator</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Alexio Mungate &amp; Anor</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Lease / Eviction</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Application for declarator opposed in the High Court</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="15" t="inlineStr">
         <is>
           <t>Round table conference on 9 April 2026</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="15" t="inlineStr">
         <is>
           <t>25/03/26</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>NGM 9A</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE-NGM9A</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Huang Li Qiang</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Civil debt and fraud claim</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Mukweva and Paswa</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Debt Collection / Fraud</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Replicated to special plea, filed heads of argument</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>Consolidate record, apply for set down date</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="J9" s="15" t="inlineStr">
         <is>
           <t>27/03/26</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>NGM 9D</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE-NGM9D</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Huang Li Qiang</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Civil claim — Cupori and Tsvere</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Cupori and Lewis Tsvere</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Debt Collection / Fraud</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="15" t="inlineStr">
         <is>
           <t>Matter removed from roll, trial postponed</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="15" t="inlineStr">
         <is>
           <t>Pursuing out of court settlement</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="15" t="inlineStr">
         <is>
           <t>31/03/26</t>
         </is>
@@ -1196,7 +1219,11 @@
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="12" t="inlineStr"/>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>NOTE: Rows 6-10 in the Matter Register sheet are EXAMPLES only. Delete them before importing, or they will be created as test matters.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="13" t="inlineStr">

</xml_diff>